<commit_message>
Billing v2 phase 8: offline counter POS (web and app WebView)
- /shop/accounts/pos: the device keeps the item list and a bill queue
  (localStorage), sends it every 15 s and on reconnect; camera scan where
  the browser has BarcodeDetector.
- GoKesari numbers each bill at sync in the order it was made (gapless);
  acc_sales_invoices.client_ref (migration 0134, seller, partial unique
  index) makes a re-sent or parallel-sent bill return the same invoice.
- Per-bill result: CREATED / DUPLICATE / REJECTED (item left the shop),
  with warnings for a changed price or stock below zero.
- Tests: scenario 16 on both layouts. Decisions D32-D33; B7 narrowed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/billing/BILLING_TRACKER_2026-11-01.xlsx
+++ b/docs/billing/BILLING_TRACKER_2026-11-01.xlsx
@@ -12,9 +12,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="198">
-  <si>
-    <t>Billing v2 tracker — updated 01-Nov-2026 IST — branch feat/billing-v2-phase1 — testing report docs/billing/TESTING_REPORT.md</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="203">
+  <si>
+    <t>Billing v2 tracker — updated 01-Nov-2026 IST (phases 1-7) — branch feat/billing-v2-phase1 — testing report docs/billing/TESTING_REPORT.md</t>
   </si>
   <si>
     <t>ID</t>
@@ -140,10 +140,16 @@
     <t>G7</t>
   </si>
   <si>
+    <t>Partial</t>
+  </si>
+  <si>
     <t>Not started</t>
   </si>
   <si>
-    <t>hsn_tax_rates exists (no UQC, not seeded)</t>
+    <t>Pass (local)</t>
+  </si>
+  <si>
+    <t>Unit→UQC map per shop (inv_unit_uqc) + export block + fix list done; HSN master seeding with UQC still open</t>
   </si>
   <si>
     <t>BV2-06</t>
@@ -158,13 +164,13 @@
     <t>G5</t>
   </si>
   <si>
-    <t>Not started (capture step)</t>
-  </si>
-  <si>
-    <t>Pass (data + engine)</t>
-  </si>
-  <si>
-    <t>Columns + backfill (0125). Next: onboarding capture, portal status from re-check</t>
+    <t>Done (engine, guard, invoice)</t>
+  </si>
+  <si>
+    <t>Pass (local, both layouts)</t>
+  </si>
+  <si>
+    <t>Columns + backfill (0125); checkout guard; invoice Enrolment ID note. Next: capture step in onboarding wizard</t>
   </si>
   <si>
     <t>BV2-07</t>
@@ -176,10 +182,7 @@
     <t>§3.3</t>
   </si>
   <si>
-    <t>Pass (engine)</t>
-  </si>
-  <si>
-    <t>Engine supplyBlock ready; checkout wiring phase 2</t>
+    <t>Checkout refuses Enrolment-ID / composition inter-state and inactive GSTINs (billing_v2)</t>
   </si>
   <si>
     <t>BV2-08</t>
@@ -206,7 +209,7 @@
     <t>G9</t>
   </si>
   <si>
-    <t>Tax invoice, bill of supply, credit note exist</t>
+    <t>acc_documents (0128): credit/debit note, receipt/refund voucher, challan, estimate; own series; books + stock; cancel; immutable</t>
   </si>
   <si>
     <t>BV2-10</t>
@@ -218,319 +221,322 @@
     <t>§4.2</t>
   </si>
   <si>
+    <t>Invoice cancellation (mark only) + immutability trigger done; numbering format still B4 (LEGACY 25 chars)</t>
+  </si>
+  <si>
+    <t>BV2-11</t>
+  </si>
+  <si>
+    <t>Mandatory invoice fields (UQC, state code, ECO GSTIN)</t>
+  </si>
+  <si>
+    <t>§4.3</t>
+  </si>
+  <si>
+    <t>Buyer GSTIN, ECO GSTIN, Enrolment ID, UQC on invoices issued under billing_v2</t>
+  </si>
+  <si>
+    <t>BV2-12</t>
+  </si>
+  <si>
+    <t>Customer B2B GSTIN at checkout with live check</t>
+  </si>
+  <si>
+    <t>§4.4</t>
+  </si>
+  <si>
+    <t>API done (checkout field UI: phase 8)</t>
+  </si>
+  <si>
+    <t>Pass (local, mock GSP)</t>
+  </si>
+  <si>
+    <t>orders.buyer_gstin (0127), format + GSP check; live check needs B1</t>
+  </si>
+  <si>
+    <t>BV2-13</t>
+  </si>
+  <si>
+    <t>Credit note on every refund, by returned line, incl. cancellation before packing</t>
+  </si>
+  <si>
+    <t>§4.5</t>
+  </si>
+  <si>
+    <t>G8</t>
+  </si>
+  <si>
+    <t>Return notes credit only returned lines; pre-packing cancellation has no invoice so no note (D17)</t>
+  </si>
+  <si>
+    <t>BV2-14</t>
+  </si>
+  <si>
+    <t>Thermal 80 mm PDF, WhatsApp share, UPI QR, JSON</t>
+  </si>
+  <si>
+    <t>§4.6</t>
+  </si>
+  <si>
+    <t>Done (API)</t>
+  </si>
+  <si>
+    <t>80 mm receipt PDF, invoice JSON, UPI QR on counter bills, WhatsApp share helper</t>
+  </si>
+  <si>
+    <t>BV2-15</t>
+  </si>
+  <si>
+    <t>POS counter billing in the same series; offline in app</t>
+  </si>
+  <si>
+    <t>§4.7</t>
+  </si>
+  <si>
+    <t>Done (WebView)</t>
+  </si>
+  <si>
+    <t>Counter POS /shop/accounts/pos: device item list + bill queue (localStorage), syncs every 15 s and on reconnect; numbers given at sync in the order bills were made (gapless), clientRef makes re-sends idempotent (migration 0134); price / stock / removed-item conflicts per bill; camera scan where the browser has BarcodeDetector. Opening the page with no network at all still needs it loaded once (no service worker) — B7.</t>
+  </si>
+  <si>
+    <t>BV2-16</t>
+  </si>
+  <si>
+    <t>s.9(5) delivery GST: rates by date, rider registration, per-order liability</t>
+  </si>
+  <si>
+    <t>§5.2</t>
+  </si>
+  <si>
+    <t>G1</t>
+  </si>
+  <si>
+    <t>GoKesari delivery-fee invoice GKS/2627/000001, catch-up sweep; behind delivery_9_5; CA to confirm (B2,B3)</t>
+  </si>
+  <si>
+    <t>BV2-17</t>
+  </si>
+  <si>
+    <t>Restaurant s.9(5) as deemed supplier</t>
+  </si>
+  <si>
+    <t>§5.3</t>
+  </si>
+  <si>
+    <t>G17</t>
+  </si>
+  <si>
+    <t>Statutory row exists (disabled)</t>
+  </si>
+  <si>
+    <t>BV2-18</t>
+  </si>
+  <si>
+    <t>TCS s.52 from money flow, per-shop ledger and certificate, GSTR-8</t>
+  </si>
+  <si>
+    <t>§5.4</t>
+  </si>
+  <si>
+    <t>G3</t>
+  </si>
+  <si>
+    <t>Money-flow-driven TCS, GSTR-8 builder + schema, per-shop statement; GSP push needs B1</t>
+  </si>
+  <si>
+    <t>BV2-19</t>
+  </si>
+  <si>
+    <t>TDS s.393: per PAN, credit-or-payout timing, Form 140 data, certificates</t>
+  </si>
+  <si>
+    <t>§5.5</t>
+  </si>
+  <si>
+    <t>G4</t>
+  </si>
+  <si>
+    <t>Per-PAN exemption, quarterly statement (Form 140 data), per-shop statement; Aadhaar-as-PAN not handled</t>
+  </si>
+  <si>
+    <t>BV2-20</t>
+  </si>
+  <si>
+    <t>Settlement ledger; monthly GoKesari fee invoice; wallet statement</t>
+  </si>
+  <si>
+    <t>§5.6</t>
+  </si>
+  <si>
+    <t>G6</t>
+  </si>
+  <si>
+    <t>Done (statements)</t>
+  </si>
+  <si>
+    <t>Wallet + settlement statements done; fee invoices stay per payout cycle (D20)</t>
+  </si>
+  <si>
+    <t>BV2-21</t>
+  </si>
+  <si>
+    <t>GoKesari's own GSTR-1 / 3B / 8, IMS, compliance dashboard</t>
+  </si>
+  <si>
+    <t>§5.7</t>
+  </si>
+  <si>
+    <t>G16</t>
+  </si>
+  <si>
+    <t>GSTR-8 / GSTR-1 (+Table 15) / 3B / TDS generate, download, mark filed; calendar + reminders; e-invoice/IMS for own purchases: phase 6</t>
+  </si>
+  <si>
+    <t>BV2-22</t>
+  </si>
+  <si>
+    <t>Shop accounting: chart of accounts, vouchers, auto-posting, reports</t>
+  </si>
+  <si>
+    <t>§6.1</t>
+  </si>
+  <si>
+    <t>G12</t>
+  </si>
+  <si>
+    <t>GoKesari activity posted into books; Tally groups; new ledgers; journal/contra/stock journal; trial balance, balance sheet, COA, TCS/TDS credit</t>
+  </si>
+  <si>
+    <t>BV2-23</t>
+  </si>
+  <si>
+    <t>Inventory: groups, godowns, transfers, reserve/dispatch, reports</t>
+  </si>
+  <si>
+    <t>§6.2</t>
+  </si>
+  <si>
+    <t>Stock journal between online/in-shop, movement + ageing reports done; more godowns, stock groups (uses categories), reserve-on-dispatch not done (D24)</t>
+  </si>
+  <si>
+    <t>BV2-24</t>
+  </si>
+  <si>
+    <t>Purchases: IRP fetch via GSP; 2B/IMS accept/reject/pending</t>
+  </si>
+  <si>
+    <t>§6.3</t>
+  </si>
+  <si>
+    <t>Done (mock GSP)</t>
+  </si>
+  <si>
+    <t>IMS accept/reject/pending pushed via GSP; supplier e-invoices → draft bill for review; live needs B1</t>
+  </si>
+  <si>
+    <t>BV2-25</t>
+  </si>
+  <si>
+    <t>Canonical model, sync log, conflict queue, masters before vouchers</t>
+  </si>
+  <si>
+    <t>§7</t>
+  </si>
+  <si>
+    <t>Canonical model, sync_records, conflict queue, masters before vouchers, validation fix list (0130)</t>
+  </si>
+  <si>
+    <t>BV2-26</t>
+  </si>
+  <si>
+    <t>File connectors: Tally Excel/.tsf/XML both ways, Busy, Marg, Vyapar, myBillBook, Zoho CSV, Odoo CSV</t>
+  </si>
+  <si>
+    <t>§8</t>
+  </si>
+  <si>
+    <t>G13, G14</t>
+  </si>
+  <si>
+    <t>Pass (local; Tally/Busy/Vyapar/myBillBook import, Tally XML round trip)</t>
+  </si>
+  <si>
+    <t>Layouts per tool; verify column maps on each tool version (B5)</t>
+  </si>
+  <si>
+    <t>BV2-27</t>
+  </si>
+  <si>
+    <t>Live connectors: Tally Windows app, Zoho OAuth, Odoo API, public REST API</t>
+  </si>
+  <si>
+    <t>G15</t>
+  </si>
+  <si>
+    <t>Tally connector 1.1.0 two-way books; connector flags; public REST API (OAuth2, scopes, OpenAPI); Zoho/Odoo adapters unchanged (invoices, credit notes, items) — contacts/bills via API not added (D28)</t>
+  </si>
+  <si>
+    <t>BV2-28</t>
+  </si>
+  <si>
+    <t>Marketplace-standard reports (MTR B2B/B2C, settlement, TCS)</t>
+  </si>
+  <si>
+    <t>G10</t>
+  </si>
+  <si>
+    <t>MTR B2B/B2C report, order-level settlement, TCS statement; monthly notice</t>
+  </si>
+  <si>
+    <t>BV2-29</t>
+  </si>
+  <si>
+    <t>Template pack and help pages (EN/HI/MR)</t>
+  </si>
+  <si>
+    <t>G13</t>
+  </si>
+  <si>
+    <t>Done (text)</t>
+  </si>
+  <si>
+    <t>Template pack + EN/HI/MR step guides; screenshots need the real software</t>
+  </si>
+  <si>
+    <t>BV2-30</t>
+  </si>
+  <si>
+    <t>GSTR-1 for shops incl. Table 14 (ECO), IFF, nil/exempt</t>
+  </si>
+  <si>
+    <t>§9.3</t>
+  </si>
+  <si>
+    <t>G11</t>
+  </si>
+  <si>
+    <t>GSTR-1 (Table 14), IFF, prepare/save/compare/file with EVC through GSP (mock); live needs B1</t>
+  </si>
+  <si>
+    <t>BV2-31</t>
+  </si>
+  <si>
+    <t>GSP connect, 2B/IMS, 3B, ledgers, e-invoice cancel, e-way bill update/cancel, CMP-08/GSTR-4, calendar</t>
+  </si>
+  <si>
+    <t>§9</t>
+  </si>
+  <si>
+    <t>G11, G16</t>
+  </si>
+  <si>
     <t>Blocked</t>
   </si>
   <si>
-    <t>B4: LEGACY default is 25 characters; owner/CA to approve GST16 from a date</t>
-  </si>
-  <si>
-    <t>BV2-11</t>
-  </si>
-  <si>
-    <t>Mandatory invoice fields (UQC, state code, ECO GSTIN)</t>
-  </si>
-  <si>
-    <t>§4.3</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>BV2-12</t>
-  </si>
-  <si>
-    <t>Customer B2B GSTIN at checkout with live check</t>
-  </si>
-  <si>
-    <t>§4.4</t>
-  </si>
-  <si>
-    <t>Live check needs GSP (B1); format check possible now</t>
-  </si>
-  <si>
-    <t>BV2-13</t>
-  </si>
-  <si>
-    <t>Credit note on every refund, by returned line, incl. cancellation before packing</t>
-  </si>
-  <si>
-    <t>§4.5</t>
-  </si>
-  <si>
-    <t>G8</t>
-  </si>
-  <si>
-    <t>Exists for delivered orders (pro-rata)</t>
-  </si>
-  <si>
-    <t>BV2-14</t>
-  </si>
-  <si>
-    <t>Thermal 80 mm PDF, WhatsApp share, UPI QR, JSON</t>
-  </si>
-  <si>
-    <t>§4.6</t>
-  </si>
-  <si>
-    <t>A4 PDF, email, B2C/IRN QR exist</t>
-  </si>
-  <si>
-    <t>BV2-15</t>
-  </si>
-  <si>
-    <t>POS counter billing in the same series; offline in app</t>
-  </si>
-  <si>
-    <t>§4.7</t>
-  </si>
-  <si>
-    <t>Partial (counter sales)</t>
-  </si>
-  <si>
-    <t>Blocked (native)</t>
-  </si>
-  <si>
-    <t>B7 for offline native</t>
-  </si>
-  <si>
-    <t>BV2-16</t>
-  </si>
-  <si>
-    <t>s.9(5) delivery GST: rates by date, rider registration, per-order liability</t>
-  </si>
-  <si>
-    <t>§5.2</t>
-  </si>
-  <si>
-    <t>G1</t>
-  </si>
-  <si>
-    <t>Pass (31 Oct 18% / 1 Nov 5% / registered rider)</t>
-  </si>
-  <si>
-    <t>Behind delivery_9_5; CA to confirm (B2, B3). Next: GoKesari delivery-fee invoice to the customer</t>
-  </si>
-  <si>
-    <t>BV2-17</t>
-  </si>
-  <si>
-    <t>Restaurant s.9(5) as deemed supplier</t>
-  </si>
-  <si>
-    <t>§5.3</t>
-  </si>
-  <si>
-    <t>G17</t>
-  </si>
-  <si>
-    <t>Statutory row exists (disabled)</t>
-  </si>
-  <si>
-    <t>BV2-18</t>
-  </si>
-  <si>
-    <t>TCS s.52 from money flow, per-shop ledger and certificate, GSTR-8</t>
-  </si>
-  <si>
-    <t>§5.4</t>
-  </si>
-  <si>
-    <t>G3</t>
-  </si>
-  <si>
-    <t>Payout TCS exists (ignores collector); GSTR-8 push needs GSP (B1)</t>
-  </si>
-  <si>
-    <t>BV2-19</t>
-  </si>
-  <si>
-    <t>TDS s.393: per PAN, credit-or-payout timing, Form 140 data, certificates</t>
-  </si>
-  <si>
-    <t>§5.5</t>
-  </si>
-  <si>
-    <t>G4</t>
-  </si>
-  <si>
-    <t>Pass (engine scope)</t>
-  </si>
-  <si>
-    <t>Payout TDS with ₹5 lakh exemption exists (per shop)</t>
-  </si>
-  <si>
-    <t>BV2-20</t>
-  </si>
-  <si>
-    <t>Settlement ledger; monthly GoKesari fee invoice; wallet statement</t>
-  </si>
-  <si>
-    <t>§5.6</t>
-  </si>
-  <si>
-    <t>G6</t>
-  </si>
-  <si>
-    <t>Partial (weekly fee invoices)</t>
-  </si>
-  <si>
-    <t>platform_invoices per payout cycle exist</t>
-  </si>
-  <si>
-    <t>BV2-21</t>
-  </si>
-  <si>
-    <t>GoKesari's own GSTR-1 / 3B / 8, IMS, compliance dashboard</t>
-  </si>
-  <si>
-    <t>§5.7</t>
-  </si>
-  <si>
-    <t>G16</t>
-  </si>
-  <si>
-    <t>Partial (GSTR-1 CSV)</t>
-  </si>
-  <si>
-    <t>B1</t>
-  </si>
-  <si>
-    <t>BV2-22</t>
-  </si>
-  <si>
-    <t>Shop accounting: chart of accounts, vouchers, auto-posting, reports</t>
-  </si>
-  <si>
-    <t>§6.1</t>
-  </si>
-  <si>
-    <t>G12</t>
-  </si>
-  <si>
-    <t>Partial</t>
-  </si>
-  <si>
-    <t>Books exist for counter sales and purchases; online orders not posted</t>
-  </si>
-  <si>
-    <t>BV2-23</t>
-  </si>
-  <si>
-    <t>Inventory: groups, godowns, transfers, reserve/dispatch, reports</t>
-  </si>
-  <si>
-    <t>§6.2</t>
-  </si>
-  <si>
-    <t>Batches, expiry, FIFO/WA exist</t>
-  </si>
-  <si>
-    <t>BV2-24</t>
-  </si>
-  <si>
-    <t>Purchases: IRP fetch via GSP; 2B/IMS accept/reject/pending</t>
-  </si>
-  <si>
-    <t>§6.3</t>
-  </si>
-  <si>
-    <t>Partial (OCR, reconciliation)</t>
-  </si>
-  <si>
-    <t>BV2-25</t>
-  </si>
-  <si>
-    <t>Canonical model, sync log, conflict queue, masters before vouchers</t>
-  </si>
-  <si>
-    <t>§7</t>
-  </si>
-  <si>
-    <t>Sync engine switched off (rule inventorySync)</t>
-  </si>
-  <si>
-    <t>BV2-26</t>
-  </si>
-  <si>
-    <t>File connectors: Tally Excel/.tsf/XML both ways, Busy, Marg, Vyapar, myBillBook, Zoho CSV, Odoo CSV</t>
-  </si>
-  <si>
-    <t>§8</t>
-  </si>
-  <si>
-    <t>G13, G14</t>
-  </si>
-  <si>
-    <t>Partial (Tally XML export, generic Excel)</t>
-  </si>
-  <si>
-    <t>BV2-27</t>
-  </si>
-  <si>
-    <t>Live connectors: Tally Windows app, Zoho OAuth, Odoo API, public REST API</t>
-  </si>
-  <si>
-    <t>G15</t>
-  </si>
-  <si>
-    <t>Partial (Tally, Zoho, Odoo exist, limited)</t>
-  </si>
-  <si>
-    <t>B5, B6</t>
-  </si>
-  <si>
-    <t>BV2-28</t>
-  </si>
-  <si>
-    <t>Marketplace-standard reports (MTR B2B/B2C, settlement, TCS)</t>
-  </si>
-  <si>
-    <t>G10</t>
-  </si>
-  <si>
-    <t>BV2-29</t>
-  </si>
-  <si>
-    <t>Template pack and help pages (EN/HI/MR)</t>
-  </si>
-  <si>
-    <t>G13</t>
-  </si>
-  <si>
-    <t>BV2-30</t>
-  </si>
-  <si>
-    <t>GSTR-1 for shops incl. Table 14 (ECO), IFF, nil/exempt</t>
-  </si>
-  <si>
-    <t>§9.3</t>
-  </si>
-  <si>
-    <t>G11</t>
-  </si>
-  <si>
-    <t>Partial (JSON/Excel without Table 14)</t>
-  </si>
-  <si>
-    <t>Filing needs GSP (B1)</t>
-  </si>
-  <si>
-    <t>BV2-31</t>
-  </si>
-  <si>
-    <t>GSP connect, 2B/IMS, 3B, ledgers, e-invoice cancel, e-way bill update/cancel, CMP-08/GSTR-4, calendar</t>
-  </si>
-  <si>
-    <t>§9</t>
-  </si>
-  <si>
-    <t>G11, G16</t>
-  </si>
-  <si>
-    <t>Partial (mock)</t>
-  </si>
-  <si>
-    <t>B1: no real GSP</t>
+    <t>Done (mock)</t>
+  </si>
+  <si>
+    <t>All §9 flows built on the mock (returns, IMS, ledgers, IRN cancel/30-day/CRN, e-way Part B/extend/cancel, CMP-08/GSTR-4, call log, retries, session reminders); live needs B1; IRN needs GST16 numbering (B4)</t>
   </si>
   <si>
     <t>BV2-32</t>
@@ -542,6 +548,9 @@
     <t>§10</t>
   </si>
   <si>
+    <t>GSP call log, OAuth secrets hashed, operators kept out of IRN/e-way writes on new routes, per-shop/client rate limits; PAN-reveal audit on TDS export</t>
+  </si>
+  <si>
     <t>BV2-33</t>
   </si>
   <si>
@@ -551,7 +560,7 @@
     <t>§14</t>
   </si>
   <si>
-    <t>B7: needs store release; web features reach the apps through the WebView</t>
+    <t>Offline POS now runs in the apps through the WebView once the page is open (BV2-15). Still B7: Bluetooth thermal printing, native scanner, opening POS cold with no network, EVC — need a store release.</t>
   </si>
   <si>
     <t>BV2-34</t>
@@ -578,7 +587,7 @@
     <t>BV2-06, BV2-07, BV2-08</t>
   </si>
   <si>
-    <t>In progress, Not started</t>
+    <t>In progress, Done, Not started</t>
   </si>
   <si>
     <t>BV2-04, BV2-05</t>
@@ -587,13 +596,13 @@
     <t>BV2-04, BV2-09, BV2-10, BV2-11, BV2-12, BV2-14, BV2-15</t>
   </si>
   <si>
-    <t>In progress, Not started, Blocked</t>
+    <t>In progress, Done</t>
   </si>
   <si>
     <t>BV2-30, BV2-31</t>
   </si>
   <si>
-    <t>Not started, Blocked</t>
+    <t>Done, Blocked</t>
   </si>
   <si>
     <t>BV2-22, BV2-25</t>
@@ -602,10 +611,16 @@
     <t>BV2-26, BV2-29</t>
   </si>
   <si>
+    <t>Done, In progress</t>
+  </si>
+  <si>
     <t>G14</t>
   </si>
   <si>
     <t>BV2-21, BV2-24, BV2-31</t>
+  </si>
+  <si>
+    <t>Done, In progress, Blocked</t>
   </si>
 </sst>
 </file>
@@ -1233,40 +1248,40 @@
       <c r="D8" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="6" t="s">
-        <v>42</v>
+      <c r="E8" s="5" t="s">
+        <v>29</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>42</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>29</v>
@@ -1275,144 +1290,144 @@
         <v>17</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>29</v>
+        <v>49</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>17</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>15</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>42</v>
+        <v>64</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>68</v>
+        <v>64</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>29</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>15</v>
@@ -1441,16 +1456,16 @@
         <v>72</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>42</v>
+        <v>64</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>22</v>
@@ -1459,7 +1474,7 @@
         <v>22</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="K14" s="3" t="s">
         <v>73</v>
@@ -1476,16 +1491,16 @@
         <v>76</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>42</v>
+        <v>64</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>42</v>
+        <v>77</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>22</v>
@@ -1494,33 +1509,33 @@
         <v>22</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>15</v>
+        <v>78</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>42</v>
+        <v>83</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>29</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>22</v>
@@ -1529,97 +1544,97 @@
         <v>22</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>42</v>
+        <v>64</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>42</v>
+        <v>64</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>90</v>
+        <v>16</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>15</v>
+        <v>51</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>29</v>
+        <v>98</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>17</v>
@@ -1634,27 +1649,27 @@
         <v>18</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>97</v>
+        <v>44</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="20" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>15</v>
@@ -1672,30 +1687,30 @@
         <v>15</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="21" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>29</v>
+        <v>108</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>17</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>22</v>
@@ -1704,33 +1719,33 @@
         <v>22</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="22" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>29</v>
+        <v>113</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>17</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>22</v>
@@ -1739,7 +1754,7 @@
         <v>22</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>113</v>
+        <v>44</v>
       </c>
       <c r="K22" s="3" t="s">
         <v>114</v>
@@ -1758,11 +1773,11 @@
       <c r="D23" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="E23" s="6" t="s">
-        <v>42</v>
+      <c r="E23" s="5" t="s">
+        <v>29</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G23" s="3" t="s">
         <v>119</v>
@@ -1774,7 +1789,7 @@
         <v>22</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="K23" s="3" t="s">
         <v>120</v>
@@ -1793,119 +1808,119 @@
       <c r="D24" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="E24" s="6" t="s">
-        <v>42</v>
+      <c r="E24" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G24" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K24" s="3" t="s">
         <v>125</v>
-      </c>
-      <c r="H24" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I24" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J24" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="K24" s="3" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="25" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="C25" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="D25" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="E25" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K25" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G25" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="H25" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I25" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J25" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="K25" s="3" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="26" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C26" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="D26" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K26" s="3" t="s">
         <v>134</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G26" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I26" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J26" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="K26" s="3" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="27" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C27" s="3" t="s">
         <v>137</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>139</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="E27" s="6" t="s">
-        <v>42</v>
+      <c r="E27" s="5" t="s">
+        <v>29</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>22</v>
@@ -1914,80 +1929,80 @@
         <v>22</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
     </row>
     <row r="28" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B28" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="C28" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="D28" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I28" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K28" s="3" t="s">
         <v>143</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G28" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="H28" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I28" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J28" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="K28" s="3" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="29" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="C29" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="D29" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="E29" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J29" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="E29" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G29" s="3" t="s">
+      <c r="K29" s="3" t="s">
         <v>149</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I29" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J29" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="K29" s="3" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="30" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1998,19 +2013,19 @@
         <v>151</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="E30" s="6" t="s">
-        <v>42</v>
+      <c r="E30" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>153</v>
+        <v>16</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>18</v>
@@ -2019,45 +2034,45 @@
         <v>18</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="31" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B31" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="C31" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="D31" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="C31" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="D31" s="3" t="s">
+      <c r="E31" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G31" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I31" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J31" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K31" s="3" t="s">
         <v>157</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G31" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="H31" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I31" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J31" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="K31" s="3" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="32" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2068,19 +2083,19 @@
         <v>159</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="E32" s="6" t="s">
-        <v>42</v>
+      <c r="E32" s="5" t="s">
+        <v>29</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>42</v>
+        <v>161</v>
       </c>
       <c r="H32" s="3" t="s">
         <v>22</v>
@@ -2092,30 +2107,30 @@
         <v>15</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>73</v>
+        <v>162</v>
       </c>
     </row>
     <row r="33" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>42</v>
+        <v>166</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>165</v>
+        <v>16</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>22</v>
@@ -2124,33 +2139,33 @@
         <v>22</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="34" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>68</v>
+        <v>172</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>22</v>
@@ -2159,30 +2174,30 @@
         <v>22</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>15</v>
+        <v>78</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="35" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E35" s="6" t="s">
-        <v>42</v>
+      <c r="E35" s="5" t="s">
+        <v>29</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G35" s="3" t="s">
         <v>15</v>
@@ -2197,24 +2212,24 @@
         <v>15</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>73</v>
+        <v>178</v>
       </c>
     </row>
     <row r="36" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>15</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>68</v>
+        <v>172</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>15</v>
@@ -2223,27 +2238,27 @@
         <v>18</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>68</v>
+        <v>172</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>68</v>
+        <v>172</v>
       </c>
       <c r="J36" s="3" t="s">
         <v>15</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="37" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>15</v>
@@ -2264,10 +2279,10 @@
         <v>15</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -2290,21 +2305,21 @@
         <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2320,35 +2335,35 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C5" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C6" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2359,7 +2374,7 @@
         <v>115</v>
       </c>
       <c r="C7" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2367,65 +2382,65 @@
         <v>41</v>
       </c>
       <c r="B8" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C8" t="s">
-        <v>188</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C9" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C10" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B12" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C12" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B13" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -2433,21 +2448,21 @@
         <v>160</v>
       </c>
       <c r="B14" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C14" t="s">
-        <v>42</v>
+        <v>199</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C15" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -2458,7 +2473,7 @@
         <v>150</v>
       </c>
       <c r="C16" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -2466,21 +2481,21 @@
         <v>124</v>
       </c>
       <c r="B17" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C17" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C18" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Billing v2: full-run results; migrate-on-build starts from a new scratch database
The test dropped the fully migrated schema in one transaction before the
"two migrations at once" case. With 0125-0135 that needs more locks than
Postgres's default lock table (max_locks_per_transaction 64, also CI's
default): building the schema takes 6,982 locks on staging's 0124 and 7,159
with 0135. The test now drops and recreates its scratch database instead;
the migrations are unchanged.

Testing report: full suite on both layouts (fc9aa17d + this fix), PDF, tracker.
The PDF script falls back to the installed Chrome when Playwright's own
Chromium build is not downloaded.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/billing/BILLING_TRACKER_2026-11-01.xlsx
+++ b/docs/billing/BILLING_TRACKER_2026-11-01.xlsx
@@ -14,7 +14,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="194">
   <si>
-    <t>Billing v2 tracker — updated 01-Nov-2026 IST (phases 1-8 + gap closure) — branch feat/billing-v2-phase1 — testing report docs/billing/TESTING_REPORT.md</t>
+    <t>Billing v2 tracker — updated 01-Nov-2026 13.45 IST (phases 1-8 + gap closure, full local run) — branch feat/billing-v2-phase1 — testing report docs/billing/TESTING_REPORT.md</t>
   </si>
   <si>
     <t>ID</t>
@@ -557,7 +557,7 @@
     <t>In progress</t>
   </si>
   <si>
-    <t>Local: pass on both layouts</t>
+    <t>Local: full suite passed on both layouts (3,248 / 3,240 + 8 skipped; only pre-existing and environment failures)</t>
   </si>
   <si>
     <t>docs/billing/TESTING_REPORT.md (+ PDF). Test and Prod sections pending the staging merge</t>

</xml_diff>